<commit_message>
Regenerate 4-table snapshot for week 28 Sep-4 Oct after Team 7/Mirkl freeze and Harlow Miller leave application. Mirkl totals updated; DBZ and KM unchanged.
</commit_message>
<xml_diff>
--- a/2026-09-28/Snapshot_4Tables_Sep28_Oct4.xlsx
+++ b/2026-09-28/Snapshot_4Tables_Sep28_Oct4.xlsx
@@ -547,7 +547,7 @@
         <v>43</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>56</v>
@@ -572,19 +572,19 @@
         <v>49</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>45</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>33</v>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>44</v>
@@ -612,7 +612,7 @@
         <v>43</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>17</v>
@@ -628,7 +628,7 @@
         <v>55</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>58</v>
@@ -637,7 +637,7 @@
         <v>63</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>42</v>
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>191</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>207</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>133</v>
@@ -710,7 +710,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+0</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>+6</t>
+          <t>+8</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>+17</t>
+          <t>+15</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1205,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>2</v>
@@ -1230,19 +1230,19 @@
         <v>3</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>4</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>2</v>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2" t="n">
         <v>3</v>
@@ -1270,7 +1270,7 @@
         <v>2</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>3</v>
@@ -1286,7 +1286,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>3</v>
@@ -1295,7 +1295,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>4</v>
@@ -1311,19 +1311,19 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C32" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>13</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>11</v>

</xml_diff>